<commit_message>
Starting to add documents and the R2 bucket was created
</commit_message>
<xml_diff>
--- a/DATA/DATA FILES/MINI SPLIT DATA.xlsx
+++ b/DATA/DATA FILES/MINI SPLIT DATA.xlsx
@@ -997,6 +997,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR7" t="inlineStr">
+        <is>
+          <t>MSBNS-H09B-1A__MO1CS-H09B-1A</t>
+        </is>
+      </c>
       <c r="BI7" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -1183,6 +1188,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>MSBNS-H09B-2A__MO1CS-H09B-2A</t>
+        </is>
+      </c>
       <c r="BI8" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -1369,6 +1379,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR9" t="inlineStr">
+        <is>
+          <t>MSBNS-H12B-1A__MO1CS-H12B-1A</t>
+        </is>
+      </c>
       <c r="BI9" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -1555,6 +1570,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR10" t="inlineStr">
+        <is>
+          <t>MSBNS-H12B-2A__MO1CS-H12B-2A</t>
+        </is>
+      </c>
       <c r="BI10" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -1741,6 +1761,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR11" t="inlineStr">
+        <is>
+          <t>MSBNS-H18B-2A__MO1CS-H18B-2A</t>
+        </is>
+      </c>
       <c r="BI11" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -1927,6 +1952,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR12" t="inlineStr">
+        <is>
+          <t>MSBNS-H24B-2A__MO1CS-H24B-2A</t>
+        </is>
+      </c>
       <c r="BI12" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -2113,6 +2143,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR13" t="inlineStr">
+        <is>
+          <t>MSBNS-H30B-2A__MO1CS-H30B-2A</t>
+        </is>
+      </c>
       <c r="BI13" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -2299,6 +2334,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR14" t="inlineStr">
+        <is>
+          <t>MSBNS-H36B-2A__MO1CS-H36B-2A</t>
+        </is>
+      </c>
       <c r="BI14" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -2485,6 +2525,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR15" t="inlineStr">
+        <is>
+          <t>MSEHU-H06B-2A__MO1HS-H06B-2A</t>
+        </is>
+      </c>
       <c r="BI15" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -2671,6 +2716,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR16" t="inlineStr">
+        <is>
+          <t>MSEHU-H09B-2A__MO1HS-H09B-2A</t>
+        </is>
+      </c>
       <c r="BI16" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -2857,6 +2907,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR17" t="inlineStr">
+        <is>
+          <t>MSEHU-H12B-2A__MO1HS-H12B-2A</t>
+        </is>
+      </c>
       <c r="BI17" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -3043,6 +3098,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR18" t="inlineStr">
+        <is>
+          <t>MSEHU-H15B-2A__MO1HS-H15B-2A</t>
+        </is>
+      </c>
       <c r="BI18" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -3229,6 +3289,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR19" t="inlineStr">
+        <is>
+          <t>MSEHU-H18B-2A__MO1HS-H18B-2A</t>
+        </is>
+      </c>
       <c r="BI19" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -3415,6 +3480,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR20" t="inlineStr">
+        <is>
+          <t>MSEHU-H24B-2A__MO1HS-H24B-2A</t>
+        </is>
+      </c>
       <c r="BI20" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -3601,6 +3671,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR21" t="inlineStr">
+        <is>
+          <t>MSEHU-H33B-2A__MO1HS-H33B-2A</t>
+        </is>
+      </c>
       <c r="BI21" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -3787,6 +3862,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR22" t="inlineStr">
+        <is>
+          <t>MSEES-H09B-1A__MO1ES-H09B-1A</t>
+        </is>
+      </c>
       <c r="BI22" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -3973,6 +4053,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR23" t="inlineStr">
+        <is>
+          <t>MSEHU-H09B-2A__MO1ES-H09B-2A</t>
+        </is>
+      </c>
       <c r="BI23" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -4159,6 +4244,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR24" t="inlineStr">
+        <is>
+          <t>MSEES-H12B-1A__MO1ES-H12B-1A</t>
+        </is>
+      </c>
       <c r="BI24" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -4345,6 +4435,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR25" t="inlineStr">
+        <is>
+          <t>MSEHU-H12B-2A__MO1ES-H12B-2A</t>
+        </is>
+      </c>
       <c r="BI25" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -4531,6 +4626,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR26" t="inlineStr">
+        <is>
+          <t>MSEEU-H15B-2A__MO1ES-H15B-2A</t>
+        </is>
+      </c>
       <c r="BI26" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -4717,6 +4817,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR27" t="inlineStr">
+        <is>
+          <t>MSEHU-H18B-2A__MO1ES-H18B-2A</t>
+        </is>
+      </c>
       <c r="BI27" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -4903,6 +5008,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR28" t="inlineStr">
+        <is>
+          <t>MSEHU-H24B-2A__MO1ES-H24B-2A</t>
+        </is>
+      </c>
       <c r="BI28" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -5089,6 +5199,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR29" t="inlineStr">
+        <is>
+          <t>MSEEU-H30B-2A__MO1BS-H30B-2A</t>
+        </is>
+      </c>
       <c r="BI29" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -5275,6 +5390,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR30" t="inlineStr">
+        <is>
+          <t>MSEEU-H36B-2A__MO1BS-H36B-2A</t>
+        </is>
+      </c>
       <c r="BI30" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -5461,6 +5581,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR31" t="inlineStr">
+        <is>
+          <t>MSESU-H06B-2A__MO1SS-H06B-2A</t>
+        </is>
+      </c>
       <c r="BI31" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -5647,6 +5772,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR32" t="inlineStr">
+        <is>
+          <t>MSESU-H09B-2A__MO1SS-H09B-2A</t>
+        </is>
+      </c>
       <c r="BI32" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -5833,6 +5963,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR33" t="inlineStr">
+        <is>
+          <t>MSESU-H12B-2A__MO1SS-H12B-2A</t>
+        </is>
+      </c>
       <c r="BI33" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -6019,6 +6154,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR34" t="inlineStr">
+        <is>
+          <t>MSESU-H18B-2A__MO1SS-H18B-2A</t>
+        </is>
+      </c>
       <c r="BI34" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -6205,6 +6345,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR35" t="inlineStr">
+        <is>
+          <t>MSGNS-H09B-1A__MO1BS-H09B-1A</t>
+        </is>
+      </c>
       <c r="BI35" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -6391,6 +6536,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR36" t="inlineStr">
+        <is>
+          <t>MSGNS-H09B-2A__MO1BS-H09B-2A</t>
+        </is>
+      </c>
       <c r="BI36" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -6577,6 +6727,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR37" t="inlineStr">
+        <is>
+          <t>MSGNS-H12B-1A__MO1BS-H12B-1A</t>
+        </is>
+      </c>
       <c r="BI37" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -6763,6 +6918,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR38" t="inlineStr">
+        <is>
+          <t>MSGNS-H12B-2A__MO1BS-H12B-2A</t>
+        </is>
+      </c>
       <c r="BI38" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -6949,6 +7109,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR39" t="inlineStr">
+        <is>
+          <t>MSGNS-H18B-2A__MO1BS-H18B-2A</t>
+        </is>
+      </c>
       <c r="BI39" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -7135,6 +7300,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR40" t="inlineStr">
+        <is>
+          <t>MSGNS-H24B-2A__MO1BS-H24B-2A</t>
+        </is>
+      </c>
       <c r="BI40" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -7321,6 +7491,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR41" t="inlineStr">
+        <is>
+          <t>MSGNS-H30B-2A__MO1BS-H30B-2A</t>
+        </is>
+      </c>
       <c r="BI41" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -7507,6 +7682,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR42" t="inlineStr">
+        <is>
+          <t>MSGNS-H36B-2A__MO1BS-H36B-2A</t>
+        </is>
+      </c>
       <c r="BI42" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -7693,6 +7873,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR43" t="inlineStr">
+        <is>
+          <t>MCAHU-H09B-2A__MO1ES-H09B-2A</t>
+        </is>
+      </c>
       <c r="BI43" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -7879,6 +8064,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR44" t="inlineStr">
+        <is>
+          <t>MCAHU-H12B-2A__MO1ES-H12B-2A</t>
+        </is>
+      </c>
       <c r="BI44" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -8065,6 +8255,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR45" t="inlineStr">
+        <is>
+          <t>MCAHU-H18B-2A__MO1ES-H18B-2A</t>
+        </is>
+      </c>
       <c r="BI45" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -8251,6 +8446,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR46" t="inlineStr">
+        <is>
+          <t>MCAHU-H06B-2A__MO1HS-H06B-2A</t>
+        </is>
+      </c>
       <c r="BI46" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -8437,6 +8637,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR47" t="inlineStr">
+        <is>
+          <t>MCAHU-H09B-2A__MO1HS-H09B-2A</t>
+        </is>
+      </c>
       <c r="BI47" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -8623,6 +8828,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR48" t="inlineStr">
+        <is>
+          <t>MCAHU-H12B-2A__MO1HS-H12B-2A</t>
+        </is>
+      </c>
       <c r="BI48" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -8809,6 +9019,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR49" t="inlineStr">
+        <is>
+          <t>MCAHU-H18B-2A__MO1HS-H18B-2A</t>
+        </is>
+      </c>
       <c r="BI49" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -8995,6 +9210,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR50" t="inlineStr">
+        <is>
+          <t>MCDHU-H09B-2A__MO1ES-H09B-2A</t>
+        </is>
+      </c>
       <c r="BI50" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -9181,6 +9401,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR51" t="inlineStr">
+        <is>
+          <t>MCDHU-H12B-2A__MO1ES-H12B-2A</t>
+        </is>
+      </c>
       <c r="BI51" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -9367,6 +9592,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR52" t="inlineStr">
+        <is>
+          <t>MCDHU-H18B-2A__MO1ES-H18B-2A</t>
+        </is>
+      </c>
       <c r="BI52" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -9553,6 +9783,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR53" t="inlineStr">
+        <is>
+          <t>MCDHU-H24B-2A__MO1ES-H24B-2A</t>
+        </is>
+      </c>
       <c r="BI53" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -9739,6 +9974,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR54" t="inlineStr">
+        <is>
+          <t>MCDHS-H36B-2A__MO1BU-H36B-2A</t>
+        </is>
+      </c>
       <c r="BI54" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -9925,6 +10165,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR55" t="inlineStr">
+        <is>
+          <t>MCDHS-H48B-2A__MO1BU-H48B-2A</t>
+        </is>
+      </c>
       <c r="BI55" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -10111,6 +10356,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR56" t="inlineStr">
+        <is>
+          <t>MCDHU-H09B-2A__MO1HS-H09B-2A</t>
+        </is>
+      </c>
       <c r="BI56" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -10297,6 +10547,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR57" t="inlineStr">
+        <is>
+          <t>MCDHU-H12B-2A__MO1HS-H12B-2A</t>
+        </is>
+      </c>
       <c r="BI57" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -10483,6 +10738,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR58" t="inlineStr">
+        <is>
+          <t>MCDHU-H18B-2A__MO1HS-H18B-2A</t>
+        </is>
+      </c>
       <c r="BI58" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -10669,6 +10929,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR59" t="inlineStr">
+        <is>
+          <t>MCDHU-H24B-2A__MO1HS-H24B-2A</t>
+        </is>
+      </c>
       <c r="BI59" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -10855,6 +11120,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR60" t="inlineStr">
+        <is>
+          <t>MCDHS-H36B-2A__MO1HU-H36B-2A</t>
+        </is>
+      </c>
       <c r="BI60" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -11041,6 +11311,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR61" t="inlineStr">
+        <is>
+          <t>MCDHS-H48B-2A__MO1HU-H48B-2A</t>
+        </is>
+      </c>
       <c r="BI61" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -11227,6 +11502,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR62" t="inlineStr">
+        <is>
+          <t>MDHHU-H09B-2A__MO1ES-H09B-2A</t>
+        </is>
+      </c>
       <c r="BI62" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -11413,6 +11693,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR63" t="inlineStr">
+        <is>
+          <t>MDLHU-H09B-2A__MO1ES-H09B-2A</t>
+        </is>
+      </c>
       <c r="BI63" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -11599,6 +11884,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR64" t="inlineStr">
+        <is>
+          <t>MDHHU-H12B-2A__MO1ES-H12B-2A</t>
+        </is>
+      </c>
       <c r="BI64" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -11785,6 +12075,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR65" t="inlineStr">
+        <is>
+          <t>MDLHU-H12B-2A__MO1ES-H12B-2A</t>
+        </is>
+      </c>
       <c r="BI65" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -11971,6 +12266,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR66" t="inlineStr">
+        <is>
+          <t>MDHHU-H18B-2A__MO1ES-H18B-2A</t>
+        </is>
+      </c>
       <c r="BI66" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -12157,6 +12457,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR67" t="inlineStr">
+        <is>
+          <t>MDLHU-H18B-2A__MO1ES-H18B-2A</t>
+        </is>
+      </c>
       <c r="BI67" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -12343,6 +12648,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR68" t="inlineStr">
+        <is>
+          <t>MDHHU-H24B-2A__MO1ES-H24B-2A</t>
+        </is>
+      </c>
       <c r="BI68" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -12529,6 +12839,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR69" t="inlineStr">
+        <is>
+          <t>MDHHS-H36B-2A__MO1BU-H36B-2A</t>
+        </is>
+      </c>
       <c r="BI69" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -12715,6 +13030,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR70" t="inlineStr">
+        <is>
+          <t>MDHHS-H48B-2A__MO1BU-H48B-2A</t>
+        </is>
+      </c>
       <c r="BI70" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -12901,6 +13221,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR71" t="inlineStr">
+        <is>
+          <t>MDHHS-H60B-2A__MO1BU-H60B-2A</t>
+        </is>
+      </c>
       <c r="BI71" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -13087,6 +13412,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR72" t="inlineStr">
+        <is>
+          <t>MDLHU-H06B-2A__MO1HS-H06B-2A</t>
+        </is>
+      </c>
       <c r="BI72" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -13273,6 +13603,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR73" t="inlineStr">
+        <is>
+          <t>MDHHU-H09B-2A__MO1HS-H09B-2A</t>
+        </is>
+      </c>
       <c r="BI73" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -13459,6 +13794,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR74" t="inlineStr">
+        <is>
+          <t>MDLHU-H09B-2A__MO1HS-H09B-2A</t>
+        </is>
+      </c>
       <c r="BI74" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -13645,6 +13985,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR75" t="inlineStr">
+        <is>
+          <t>MDHHU-H12B-2A__MO1HS-H12B-2A</t>
+        </is>
+      </c>
       <c r="BI75" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -13831,6 +14176,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR76" t="inlineStr">
+        <is>
+          <t>MDLHU-H12B-2A__MO1HS-H12B-2A</t>
+        </is>
+      </c>
       <c r="BI76" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -14017,6 +14367,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR77" t="inlineStr">
+        <is>
+          <t>MDHHU-H18B-2A__MO1HS-H18B-2A</t>
+        </is>
+      </c>
       <c r="BI77" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -14203,6 +14558,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR78" t="inlineStr">
+        <is>
+          <t>MDLHU-H18B-2A__MO1HS-H18B-2A</t>
+        </is>
+      </c>
       <c r="BI78" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -14389,6 +14749,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR79" t="inlineStr">
+        <is>
+          <t>MDHHU-H24B-2A__MO1HS-H24B-2A</t>
+        </is>
+      </c>
       <c r="BI79" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -14575,6 +14940,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR80" t="inlineStr">
+        <is>
+          <t>MDHHS-H36B-2A__MO1HU-H36B-2A</t>
+        </is>
+      </c>
       <c r="BI80" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -14761,6 +15131,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR81" t="inlineStr">
+        <is>
+          <t>MDHHS-H48B-2A__MO1HU-H48B-2A</t>
+        </is>
+      </c>
       <c r="BI81" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -14947,6 +15322,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR82" t="inlineStr">
+        <is>
+          <t>MDHHS-H60B-2A__MO1HU-H60B-2A</t>
+        </is>
+      </c>
       <c r="BI82" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -15133,6 +15513,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR83" t="inlineStr">
+        <is>
+          <t>MFAHU-H09B-2A__MO1ES-H09B-2A</t>
+        </is>
+      </c>
       <c r="BI83" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -15319,6 +15704,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR84" t="inlineStr">
+        <is>
+          <t>MFAHU-H12B-2A__MO1ES-H12B-2A</t>
+        </is>
+      </c>
       <c r="BI84" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -15505,6 +15895,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR85" t="inlineStr">
+        <is>
+          <t>MFAHU-H16B-2A__MO1ES-H18B-2A</t>
+        </is>
+      </c>
       <c r="BI85" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -15691,6 +16086,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR86" t="inlineStr">
+        <is>
+          <t>MFAHU-H09B-2A__MO1HS-H09B-2A</t>
+        </is>
+      </c>
       <c r="BI86" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -15877,6 +16277,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR87" t="inlineStr">
+        <is>
+          <t>MFAHU-H12B-2A__MO1HS-H12B-2A</t>
+        </is>
+      </c>
       <c r="BI87" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -16063,6 +16468,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR88" t="inlineStr">
+        <is>
+          <t>MFAHU-H16B-2A__MO1HS-H18B-2A</t>
+        </is>
+      </c>
       <c r="BI88" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -16249,6 +16659,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR89" t="inlineStr">
+        <is>
+          <t>MFBHU-H18B-2A__MO1ES-H18B-2A</t>
+        </is>
+      </c>
       <c r="BI89" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -16435,6 +16850,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR90" t="inlineStr">
+        <is>
+          <t>MFBHU-H24B-2A__MO1ES-H24B-2A</t>
+        </is>
+      </c>
       <c r="BI90" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -16621,6 +17041,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR91" t="inlineStr">
+        <is>
+          <t>MFBHS-H36B-2A__MO1BU-H36B-2A</t>
+        </is>
+      </c>
       <c r="BI91" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -16807,6 +17232,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR92" t="inlineStr">
+        <is>
+          <t>MFBHS-H60B-2A__MO1BU-H60B-2A</t>
+        </is>
+      </c>
       <c r="BI92" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -16993,6 +17423,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR93" t="inlineStr">
+        <is>
+          <t>MFBHU-H18B-2A__MO1HS-H18B-2A</t>
+        </is>
+      </c>
       <c r="BI93" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -17179,6 +17614,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR94" t="inlineStr">
+        <is>
+          <t>MFBHU-H24B-2A__MO1HS-H24B-2A</t>
+        </is>
+      </c>
       <c r="BI94" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -17365,6 +17805,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR95" t="inlineStr">
+        <is>
+          <t>MFBHS-H36B-2A__MO1HU-H36B-2A</t>
+        </is>
+      </c>
       <c r="BI95" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -17551,6 +17996,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR96" t="inlineStr">
+        <is>
+          <t>MFBHS-H48B-2A__MO1HU-H48B-2A</t>
+        </is>
+      </c>
       <c r="BI96" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -17737,6 +18187,11 @@
           <t>-</t>
         </is>
       </c>
+      <c r="AR97" t="inlineStr">
+        <is>
+          <t>MFBHS-H60B-2A__MO1HU-H60B-2A</t>
+        </is>
+      </c>
       <c r="BI97" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -17921,6 +18376,11 @@
       <c r="AN98" t="inlineStr">
         <is>
           <t>-</t>
+        </is>
+      </c>
+      <c r="AR98" t="inlineStr">
+        <is>
+          <t>MFBHS-H48B-2A__MO1BU-H48B-2A</t>
         </is>
       </c>
       <c r="BI98" t="inlineStr">

</xml_diff>

<commit_message>
Adding IOM for Midea
</commit_message>
<xml_diff>
--- a/DATA/DATA FILES/MINI SPLIT DATA.xlsx
+++ b/DATA/DATA FILES/MINI SPLIT DATA.xlsx
@@ -560,12 +560,12 @@
       </c>
       <c r="AT2" s="1" t="inlineStr">
         <is>
-          <t>ENGINEERING MANUAL (OUTDOOR UNIT)</t>
+          <t>SERVICE MANUAL (OUTDOOR UNIT)</t>
         </is>
       </c>
       <c r="AU2" s="1" t="inlineStr">
         <is>
-          <t>ENGINEERING MANUAL (INDOOR UNIT)</t>
+          <t>SERVICE MANUAL (INDOOR UNIT)</t>
         </is>
       </c>
       <c r="AV2" s="1" t="inlineStr">
@@ -1002,6 +1002,16 @@
           <t>MSBNS-H09B-1A__MO1CS-H09B-1A</t>
         </is>
       </c>
+      <c r="AU7" t="inlineStr">
+        <is>
+          <t>Midea Infinite Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY7" t="inlineStr">
+        <is>
+          <t>Midea MSBNS Infini L Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI7" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -1193,6 +1203,16 @@
           <t>MSBNS-H09B-2A__MO1CS-H09B-2A</t>
         </is>
       </c>
+      <c r="AU8" t="inlineStr">
+        <is>
+          <t>Midea Infinite Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY8" t="inlineStr">
+        <is>
+          <t>Midea MSBNS Infini L Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI8" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -1384,6 +1404,16 @@
           <t>MSBNS-H12B-1A__MO1CS-H12B-1A</t>
         </is>
       </c>
+      <c r="AU9" t="inlineStr">
+        <is>
+          <t>Midea Infinite Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY9" t="inlineStr">
+        <is>
+          <t>Midea MSBNS Infini L Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI9" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -1575,6 +1605,16 @@
           <t>MSBNS-H12B-2A__MO1CS-H12B-2A</t>
         </is>
       </c>
+      <c r="AU10" t="inlineStr">
+        <is>
+          <t>Midea Infinite Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY10" t="inlineStr">
+        <is>
+          <t>Midea MSBNS Infini L Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI10" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -1766,6 +1806,16 @@
           <t>MSBNS-H18B-2A__MO1CS-H18B-2A</t>
         </is>
       </c>
+      <c r="AU11" t="inlineStr">
+        <is>
+          <t>Midea Infinite Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY11" t="inlineStr">
+        <is>
+          <t>Midea MSBNS Infini L Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI11" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -1957,6 +2007,16 @@
           <t>MSBNS-H24B-2A__MO1CS-H24B-2A</t>
         </is>
       </c>
+      <c r="AU12" t="inlineStr">
+        <is>
+          <t>Midea Infinite Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY12" t="inlineStr">
+        <is>
+          <t>Midea MSBNS Infini L Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI12" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -2148,6 +2208,16 @@
           <t>MSBNS-H30B-2A__MO1CS-H30B-2A</t>
         </is>
       </c>
+      <c r="AU13" t="inlineStr">
+        <is>
+          <t>Midea Infinite Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY13" t="inlineStr">
+        <is>
+          <t>Midea MSBNS Infini L Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI13" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -2339,6 +2409,16 @@
           <t>MSBNS-H36B-2A__MO1CS-H36B-2A</t>
         </is>
       </c>
+      <c r="AU14" t="inlineStr">
+        <is>
+          <t>Midea Infinite Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY14" t="inlineStr">
+        <is>
+          <t>Midea MSBNS Infini L Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI14" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -2530,6 +2610,21 @@
           <t>MSEHU-H06B-2A__MO1HS-H06B-2A</t>
         </is>
       </c>
+      <c r="AT15" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU15" t="inlineStr">
+        <is>
+          <t>Midea All Easy Pro Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY15" t="inlineStr">
+        <is>
+          <t>Midea MSEHU-MSEES-MSEEU All Easy Pro Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI15" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -2721,6 +2816,21 @@
           <t>MSEHU-H09B-2A__MO1HS-H09B-2A</t>
         </is>
       </c>
+      <c r="AT16" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU16" t="inlineStr">
+        <is>
+          <t>Midea All Easy Pro Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY16" t="inlineStr">
+        <is>
+          <t>Midea MSEHU-MSEES-MSEEU All Easy Pro Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI16" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -2912,6 +3022,21 @@
           <t>MSEHU-H12B-2A__MO1HS-H12B-2A</t>
         </is>
       </c>
+      <c r="AT17" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU17" t="inlineStr">
+        <is>
+          <t>Midea All Easy Pro Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY17" t="inlineStr">
+        <is>
+          <t>Midea MSEHU-MSEES-MSEEU All Easy Pro Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI17" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -3103,6 +3228,21 @@
           <t>MSEHU-H15B-2A__MO1HS-H15B-2A</t>
         </is>
       </c>
+      <c r="AT18" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU18" t="inlineStr">
+        <is>
+          <t>Midea All Easy Pro Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY18" t="inlineStr">
+        <is>
+          <t>Midea MSEHU-MSEES-MSEEU All Easy Pro Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI18" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -3294,6 +3434,21 @@
           <t>MSEHU-H18B-2A__MO1HS-H18B-2A</t>
         </is>
       </c>
+      <c r="AT19" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU19" t="inlineStr">
+        <is>
+          <t>Midea All Easy Pro Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY19" t="inlineStr">
+        <is>
+          <t>Midea MSEHU-MSEES-MSEEU All Easy Pro Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI19" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -3485,6 +3640,21 @@
           <t>MSEHU-H24B-2A__MO1HS-H24B-2A</t>
         </is>
       </c>
+      <c r="AT20" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU20" t="inlineStr">
+        <is>
+          <t>Midea All Easy Pro Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY20" t="inlineStr">
+        <is>
+          <t>Midea MSEHU-MSEES-MSEEU All Easy Pro Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI20" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -3676,6 +3846,21 @@
           <t>MSEHU-H33B-2A__MO1HS-H33B-2A</t>
         </is>
       </c>
+      <c r="AT21" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU21" t="inlineStr">
+        <is>
+          <t>Midea All Easy Pro Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY21" t="inlineStr">
+        <is>
+          <t>Midea MSEHU-MSEES-MSEEU All Easy Pro Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI21" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -3867,6 +4052,21 @@
           <t>MSEES-H09B-1A__MO1ES-H09B-1A</t>
         </is>
       </c>
+      <c r="AT22" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU22" t="inlineStr">
+        <is>
+          <t>Midea All Easy Pro Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY22" t="inlineStr">
+        <is>
+          <t>Midea MSEHU-MSEES-MSEEU All Easy Pro Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI22" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -4058,6 +4258,21 @@
           <t>MSEHU-H09B-2A__MO1ES-H09B-2A</t>
         </is>
       </c>
+      <c r="AT23" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU23" t="inlineStr">
+        <is>
+          <t>Midea All Easy Pro Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY23" t="inlineStr">
+        <is>
+          <t>Midea MSEHU-MSEES-MSEEU All Easy Pro Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI23" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -4249,6 +4464,21 @@
           <t>MSEES-H12B-1A__MO1ES-H12B-1A</t>
         </is>
       </c>
+      <c r="AT24" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU24" t="inlineStr">
+        <is>
+          <t>Midea All Easy Pro Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY24" t="inlineStr">
+        <is>
+          <t>Midea MSEHU-MSEES-MSEEU All Easy Pro Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI24" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -4440,6 +4670,21 @@
           <t>MSEHU-H12B-2A__MO1ES-H12B-2A</t>
         </is>
       </c>
+      <c r="AT25" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU25" t="inlineStr">
+        <is>
+          <t>Midea All Easy Pro Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY25" t="inlineStr">
+        <is>
+          <t>Midea MSEHU-MSEES-MSEEU All Easy Pro Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI25" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -4631,6 +4876,21 @@
           <t>MSEEU-H15B-2A__MO1ES-H15B-2A</t>
         </is>
       </c>
+      <c r="AT26" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU26" t="inlineStr">
+        <is>
+          <t>Midea All Easy Pro Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY26" t="inlineStr">
+        <is>
+          <t>Midea MSEHU-MSEES-MSEEU All Easy Pro Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI26" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -4822,6 +5082,21 @@
           <t>MSEHU-H18B-2A__MO1ES-H18B-2A</t>
         </is>
       </c>
+      <c r="AT27" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU27" t="inlineStr">
+        <is>
+          <t>Midea All Easy Pro Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY27" t="inlineStr">
+        <is>
+          <t>Midea MSEHU-MSEES-MSEEU All Easy Pro Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI27" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -5013,6 +5288,21 @@
           <t>MSEHU-H24B-2A__MO1ES-H24B-2A</t>
         </is>
       </c>
+      <c r="AT28" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU28" t="inlineStr">
+        <is>
+          <t>Midea All Easy Pro Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY28" t="inlineStr">
+        <is>
+          <t>Midea MSEHU-MSEES-MSEEU All Easy Pro Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI28" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -5204,6 +5494,21 @@
           <t>MSEEU-H30B-2A__MO1BS-H30B-2A</t>
         </is>
       </c>
+      <c r="AT29" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU29" t="inlineStr">
+        <is>
+          <t>Midea All Easy Pro Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY29" t="inlineStr">
+        <is>
+          <t>Midea MSEHU-MSEES-MSEEU All Easy Pro Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI29" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -5395,6 +5700,21 @@
           <t>MSEEU-H36B-2A__MO1BS-H36B-2A</t>
         </is>
       </c>
+      <c r="AT30" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU30" t="inlineStr">
+        <is>
+          <t>Midea All Easy Pro Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY30" t="inlineStr">
+        <is>
+          <t>Midea MSEHU-MSEES-MSEEU All Easy Pro Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI30" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -5586,6 +5906,16 @@
           <t>MSESU-H06B-2A__MO1SS-H06B-2A</t>
         </is>
       </c>
+      <c r="AU31" t="inlineStr">
+        <is>
+          <t>Midea All Easy Pro Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY31" t="inlineStr">
+        <is>
+          <t>Midea MSESU All Easy Pro High End Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI31" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -5777,6 +6107,16 @@
           <t>MSESU-H09B-2A__MO1SS-H09B-2A</t>
         </is>
       </c>
+      <c r="AU32" t="inlineStr">
+        <is>
+          <t>Midea All Easy Pro Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY32" t="inlineStr">
+        <is>
+          <t>Midea MSESU All Easy Pro High End Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI32" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -5968,6 +6308,16 @@
           <t>MSESU-H12B-2A__MO1SS-H12B-2A</t>
         </is>
       </c>
+      <c r="AU33" t="inlineStr">
+        <is>
+          <t>Midea All Easy Pro Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY33" t="inlineStr">
+        <is>
+          <t>Midea MSESU All Easy Pro High End Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI33" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -6159,6 +6509,16 @@
           <t>MSESU-H18B-2A__MO1SS-H18B-2A</t>
         </is>
       </c>
+      <c r="AU34" t="inlineStr">
+        <is>
+          <t>Midea All Easy Pro Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY34" t="inlineStr">
+        <is>
+          <t>Midea MSESU All Easy Pro High End Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI34" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -6350,6 +6710,21 @@
           <t>MSGNS-H09B-1A__MO1BS-H09B-1A</t>
         </is>
       </c>
+      <c r="AT35" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU35" t="inlineStr">
+        <is>
+          <t>Midea Infinite Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY35" t="inlineStr">
+        <is>
+          <t>Midea MSGNS Infinite Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI35" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -6541,6 +6916,21 @@
           <t>MSGNS-H09B-2A__MO1BS-H09B-2A</t>
         </is>
       </c>
+      <c r="AT36" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU36" t="inlineStr">
+        <is>
+          <t>Midea Infinite Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY36" t="inlineStr">
+        <is>
+          <t>Midea MSGNS Infinite Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI36" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -6732,6 +7122,21 @@
           <t>MSGNS-H12B-1A__MO1BS-H12B-1A</t>
         </is>
       </c>
+      <c r="AT37" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU37" t="inlineStr">
+        <is>
+          <t>Midea Infinite Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY37" t="inlineStr">
+        <is>
+          <t>Midea MSGNS Infinite Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI37" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -6923,6 +7328,21 @@
           <t>MSGNS-H12B-2A__MO1BS-H12B-2A</t>
         </is>
       </c>
+      <c r="AT38" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU38" t="inlineStr">
+        <is>
+          <t>Midea Infinite Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY38" t="inlineStr">
+        <is>
+          <t>Midea MSGNS Infinite Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI38" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -7114,6 +7534,21 @@
           <t>MSGNS-H18B-2A__MO1BS-H18B-2A</t>
         </is>
       </c>
+      <c r="AT39" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU39" t="inlineStr">
+        <is>
+          <t>Midea Infinite Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY39" t="inlineStr">
+        <is>
+          <t>Midea MSGNS Infinite Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI39" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -7305,6 +7740,21 @@
           <t>MSGNS-H24B-2A__MO1BS-H24B-2A</t>
         </is>
       </c>
+      <c r="AT40" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU40" t="inlineStr">
+        <is>
+          <t>Midea Infinite Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY40" t="inlineStr">
+        <is>
+          <t>Midea MSGNS Infinite Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI40" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -7496,6 +7946,21 @@
           <t>MSGNS-H30B-2A__MO1BS-H30B-2A</t>
         </is>
       </c>
+      <c r="AT41" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU41" t="inlineStr">
+        <is>
+          <t>Midea Infinite Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY41" t="inlineStr">
+        <is>
+          <t>Midea MSGNS Infinite Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI41" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -7687,6 +8152,21 @@
           <t>MSGNS-H36B-2A__MO1BS-H36B-2A</t>
         </is>
       </c>
+      <c r="AT42" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU42" t="inlineStr">
+        <is>
+          <t>Midea Infinite Wall Mounted Service Manual</t>
+        </is>
+      </c>
+      <c r="AY42" t="inlineStr">
+        <is>
+          <t>Midea MSGNS Infinite Wall Mounted Installation Manual</t>
+        </is>
+      </c>
       <c r="BI42" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -7878,6 +8358,26 @@
           <t>MCAHU-H09B-2A__MO1ES-H09B-2A</t>
         </is>
       </c>
+      <c r="AT43" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU43" t="inlineStr">
+        <is>
+          <t>Midea One-Way Cassette Service Manual</t>
+        </is>
+      </c>
+      <c r="AY43" t="inlineStr">
+        <is>
+          <t>Midea MCAHU One-Way Cassette Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG43" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI43" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -8069,6 +8569,26 @@
           <t>MCAHU-H12B-2A__MO1ES-H12B-2A</t>
         </is>
       </c>
+      <c r="AT44" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU44" t="inlineStr">
+        <is>
+          <t>Midea One-Way Cassette Service Manual</t>
+        </is>
+      </c>
+      <c r="AY44" t="inlineStr">
+        <is>
+          <t>Midea MCAHU One-Way Cassette Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG44" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI44" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -8260,6 +8780,26 @@
           <t>MCAHU-H18B-2A__MO1ES-H18B-2A</t>
         </is>
       </c>
+      <c r="AT45" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU45" t="inlineStr">
+        <is>
+          <t>Midea One-Way Cassette Service Manual</t>
+        </is>
+      </c>
+      <c r="AY45" t="inlineStr">
+        <is>
+          <t>Midea MCAHU One-Way Cassette Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG45" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI45" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -8451,6 +8991,26 @@
           <t>MCAHU-H06B-2A__MO1HS-H06B-2A</t>
         </is>
       </c>
+      <c r="AT46" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU46" t="inlineStr">
+        <is>
+          <t>Midea One-Way Cassette Service Manual</t>
+        </is>
+      </c>
+      <c r="AY46" t="inlineStr">
+        <is>
+          <t>Midea MCAHU One-Way Cassette Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG46" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI46" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -8642,6 +9202,26 @@
           <t>MCAHU-H09B-2A__MO1HS-H09B-2A</t>
         </is>
       </c>
+      <c r="AT47" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU47" t="inlineStr">
+        <is>
+          <t>Midea One-Way Cassette Service Manual</t>
+        </is>
+      </c>
+      <c r="AY47" t="inlineStr">
+        <is>
+          <t>Midea MCAHU One-Way Cassette Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG47" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI47" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -8833,6 +9413,26 @@
           <t>MCAHU-H12B-2A__MO1HS-H12B-2A</t>
         </is>
       </c>
+      <c r="AT48" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU48" t="inlineStr">
+        <is>
+          <t>Midea One-Way Cassette Service Manual</t>
+        </is>
+      </c>
+      <c r="AY48" t="inlineStr">
+        <is>
+          <t>Midea MCAHU One-Way Cassette Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG48" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI48" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -9024,6 +9624,26 @@
           <t>MCAHU-H18B-2A__MO1HS-H18B-2A</t>
         </is>
       </c>
+      <c r="AT49" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU49" t="inlineStr">
+        <is>
+          <t>Midea One-Way Cassette Service Manual</t>
+        </is>
+      </c>
+      <c r="AY49" t="inlineStr">
+        <is>
+          <t>Midea MCAHU One-Way Cassette Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG49" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI49" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -9215,6 +9835,26 @@
           <t>MCDHU-H09B-2A__MO1ES-H09B-2A</t>
         </is>
       </c>
+      <c r="AT50" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU50" t="inlineStr">
+        <is>
+          <t>Midea Four-Way Cassette Service Manual</t>
+        </is>
+      </c>
+      <c r="AY50" t="inlineStr">
+        <is>
+          <t>Midea MCDHU-MCDHS Compact Round Flow Cassette Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG50" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI50" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -9406,6 +10046,26 @@
           <t>MCDHU-H12B-2A__MO1ES-H12B-2A</t>
         </is>
       </c>
+      <c r="AT51" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU51" t="inlineStr">
+        <is>
+          <t>Midea Four-Way Cassette Service Manual</t>
+        </is>
+      </c>
+      <c r="AY51" t="inlineStr">
+        <is>
+          <t>Midea MCDHU-MCDHS Compact Round Flow Cassette Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG51" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI51" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -9597,6 +10257,26 @@
           <t>MCDHU-H18B-2A__MO1ES-H18B-2A</t>
         </is>
       </c>
+      <c r="AT52" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU52" t="inlineStr">
+        <is>
+          <t>Midea Four-Way Cassette Service Manual</t>
+        </is>
+      </c>
+      <c r="AY52" t="inlineStr">
+        <is>
+          <t>Midea MCDHU-MCDHS Compact Round Flow Cassette Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG52" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI52" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -9788,6 +10468,26 @@
           <t>MCDHU-H24B-2A__MO1ES-H24B-2A</t>
         </is>
       </c>
+      <c r="AT53" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU53" t="inlineStr">
+        <is>
+          <t>Midea Four-Way Cassette Service Manual</t>
+        </is>
+      </c>
+      <c r="AY53" t="inlineStr">
+        <is>
+          <t>Midea MCDHU-MCDHS Compact Round Flow Cassette Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG53" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI53" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -9979,6 +10679,26 @@
           <t>MCDHS-H36B-2A__MO1BU-H36B-2A</t>
         </is>
       </c>
+      <c r="AT54" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU54" t="inlineStr">
+        <is>
+          <t>Midea Four-Way Cassette Service Manual</t>
+        </is>
+      </c>
+      <c r="AY54" t="inlineStr">
+        <is>
+          <t>Midea MCDHU-MCDHS Compact Round Flow Cassette Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG54" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI54" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -10170,6 +10890,26 @@
           <t>MCDHS-H48B-2A__MO1BU-H48B-2A</t>
         </is>
       </c>
+      <c r="AT55" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU55" t="inlineStr">
+        <is>
+          <t>Midea Four-Way Cassette Service Manual</t>
+        </is>
+      </c>
+      <c r="AY55" t="inlineStr">
+        <is>
+          <t>Midea MCDHU-MCDHS Compact Round Flow Cassette Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG55" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI55" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -10361,6 +11101,26 @@
           <t>MCDHU-H09B-2A__MO1HS-H09B-2A</t>
         </is>
       </c>
+      <c r="AT56" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU56" t="inlineStr">
+        <is>
+          <t>Midea Four-Way Cassette Service Manual</t>
+        </is>
+      </c>
+      <c r="AY56" t="inlineStr">
+        <is>
+          <t>Midea MCDHU-MCDHS Compact Round Flow Cassette Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG56" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI56" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -10552,6 +11312,26 @@
           <t>MCDHU-H12B-2A__MO1HS-H12B-2A</t>
         </is>
       </c>
+      <c r="AT57" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU57" t="inlineStr">
+        <is>
+          <t>Midea Four-Way Cassette Service Manual</t>
+        </is>
+      </c>
+      <c r="AY57" t="inlineStr">
+        <is>
+          <t>Midea MCDHU-MCDHS Compact Round Flow Cassette Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG57" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI57" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -10743,6 +11523,26 @@
           <t>MCDHU-H18B-2A__MO1HS-H18B-2A</t>
         </is>
       </c>
+      <c r="AT58" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU58" t="inlineStr">
+        <is>
+          <t>Midea Four-Way Cassette Service Manual</t>
+        </is>
+      </c>
+      <c r="AY58" t="inlineStr">
+        <is>
+          <t>Midea MCDHU-MCDHS Compact Round Flow Cassette Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG58" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI58" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -10934,6 +11734,26 @@
           <t>MCDHU-H24B-2A__MO1HS-H24B-2A</t>
         </is>
       </c>
+      <c r="AT59" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU59" t="inlineStr">
+        <is>
+          <t>Midea Four-Way Cassette Service Manual</t>
+        </is>
+      </c>
+      <c r="AY59" t="inlineStr">
+        <is>
+          <t>Midea MCDHU-MCDHS Compact Round Flow Cassette Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG59" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI59" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -11125,6 +11945,26 @@
           <t>MCDHS-H36B-2A__MO1HU-H36B-2A</t>
         </is>
       </c>
+      <c r="AT60" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU60" t="inlineStr">
+        <is>
+          <t>Midea Four-Way Cassette Service Manual</t>
+        </is>
+      </c>
+      <c r="AY60" t="inlineStr">
+        <is>
+          <t>Midea MCDHU-MCDHS Compact Round Flow Cassette Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG60" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI60" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -11316,6 +12156,26 @@
           <t>MCDHS-H48B-2A__MO1HU-H48B-2A</t>
         </is>
       </c>
+      <c r="AT61" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU61" t="inlineStr">
+        <is>
+          <t>Midea Four-Way Cassette Service Manual</t>
+        </is>
+      </c>
+      <c r="AY61" t="inlineStr">
+        <is>
+          <t>Midea MCDHU-MCDHS Compact Round Flow Cassette Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG61" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI61" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -11507,6 +12367,26 @@
           <t>MDHHU-H09B-2A__MO1ES-H09B-2A</t>
         </is>
       </c>
+      <c r="AT62" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU62" t="inlineStr">
+        <is>
+          <t>Midea High Static Duct Service Manual</t>
+        </is>
+      </c>
+      <c r="AY62" t="inlineStr">
+        <is>
+          <t>Midea MDHHU-MDHHS High Static Duct Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG62" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI62" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -11698,6 +12578,26 @@
           <t>MDLHU-H09B-2A__MO1ES-H09B-2A</t>
         </is>
       </c>
+      <c r="AT63" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU63" t="inlineStr">
+        <is>
+          <t>Midea Low Static Duct Service Manual</t>
+        </is>
+      </c>
+      <c r="AY63" t="inlineStr">
+        <is>
+          <t>Midea MDLHU Low Static Slim Duct Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG63" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI63" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -11889,6 +12789,26 @@
           <t>MDHHU-H12B-2A__MO1ES-H12B-2A</t>
         </is>
       </c>
+      <c r="AT64" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU64" t="inlineStr">
+        <is>
+          <t>Midea High Static Duct Service Manual</t>
+        </is>
+      </c>
+      <c r="AY64" t="inlineStr">
+        <is>
+          <t>Midea MDHHU-MDHHS High Static Duct Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG64" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI64" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -12080,6 +13000,26 @@
           <t>MDLHU-H12B-2A__MO1ES-H12B-2A</t>
         </is>
       </c>
+      <c r="AT65" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU65" t="inlineStr">
+        <is>
+          <t>Midea Low Static Duct Service Manual</t>
+        </is>
+      </c>
+      <c r="AY65" t="inlineStr">
+        <is>
+          <t>Midea MDLHU Low Static Slim Duct Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG65" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI65" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -12271,6 +13211,26 @@
           <t>MDHHU-H18B-2A__MO1ES-H18B-2A</t>
         </is>
       </c>
+      <c r="AT66" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU66" t="inlineStr">
+        <is>
+          <t>Midea High Static Duct Service Manual</t>
+        </is>
+      </c>
+      <c r="AY66" t="inlineStr">
+        <is>
+          <t>Midea MDHHU-MDHHS High Static Duct Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG66" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI66" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -12462,6 +13422,26 @@
           <t>MDLHU-H18B-2A__MO1ES-H18B-2A</t>
         </is>
       </c>
+      <c r="AT67" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU67" t="inlineStr">
+        <is>
+          <t>Midea Low Static Duct Service Manual</t>
+        </is>
+      </c>
+      <c r="AY67" t="inlineStr">
+        <is>
+          <t>Midea MDLHU Low Static Slim Duct Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG67" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI67" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -12653,6 +13633,26 @@
           <t>MDHHU-H24B-2A__MO1ES-H24B-2A</t>
         </is>
       </c>
+      <c r="AT68" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU68" t="inlineStr">
+        <is>
+          <t>Midea High Static Duct Service Manual</t>
+        </is>
+      </c>
+      <c r="AY68" t="inlineStr">
+        <is>
+          <t>Midea MDHHU-MDHHS High Static Duct Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG68" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI68" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -12844,6 +13844,26 @@
           <t>MDHHS-H36B-2A__MO1BU-H36B-2A</t>
         </is>
       </c>
+      <c r="AT69" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU69" t="inlineStr">
+        <is>
+          <t>Midea High Static Duct Service Manual</t>
+        </is>
+      </c>
+      <c r="AY69" t="inlineStr">
+        <is>
+          <t>Midea MDHHU-MDHHS High Static Duct Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG69" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI69" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -13035,6 +14055,26 @@
           <t>MDHHS-H48B-2A__MO1BU-H48B-2A</t>
         </is>
       </c>
+      <c r="AT70" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU70" t="inlineStr">
+        <is>
+          <t>Midea High Static Duct Service Manual</t>
+        </is>
+      </c>
+      <c r="AY70" t="inlineStr">
+        <is>
+          <t>Midea MDHHU-MDHHS High Static Duct Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG70" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI70" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -13226,6 +14266,26 @@
           <t>MDHHS-H60B-2A__MO1BU-H60B-2A</t>
         </is>
       </c>
+      <c r="AT71" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU71" t="inlineStr">
+        <is>
+          <t>Midea High Static Duct Service Manual</t>
+        </is>
+      </c>
+      <c r="AY71" t="inlineStr">
+        <is>
+          <t>Midea MDHHU-MDHHS High Static Duct Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG71" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI71" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -13417,6 +14477,26 @@
           <t>MDLHU-H06B-2A__MO1HS-H06B-2A</t>
         </is>
       </c>
+      <c r="AT72" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU72" t="inlineStr">
+        <is>
+          <t>Midea Low Static Duct Service Manual</t>
+        </is>
+      </c>
+      <c r="AY72" t="inlineStr">
+        <is>
+          <t>Midea MDLHU Low Static Slim Duct Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG72" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI72" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -13608,6 +14688,26 @@
           <t>MDHHU-H09B-2A__MO1HS-H09B-2A</t>
         </is>
       </c>
+      <c r="AT73" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU73" t="inlineStr">
+        <is>
+          <t>Midea High Static Duct Service Manual</t>
+        </is>
+      </c>
+      <c r="AY73" t="inlineStr">
+        <is>
+          <t>Midea MDHHU-MDHHS High Static Duct Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG73" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI73" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -13799,6 +14899,26 @@
           <t>MDLHU-H09B-2A__MO1HS-H09B-2A</t>
         </is>
       </c>
+      <c r="AT74" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU74" t="inlineStr">
+        <is>
+          <t>Midea Low Static Duct Service Manual</t>
+        </is>
+      </c>
+      <c r="AY74" t="inlineStr">
+        <is>
+          <t>Midea MDLHU Low Static Slim Duct Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG74" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI74" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -13990,6 +15110,26 @@
           <t>MDHHU-H12B-2A__MO1HS-H12B-2A</t>
         </is>
       </c>
+      <c r="AT75" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU75" t="inlineStr">
+        <is>
+          <t>Midea High Static Duct Service Manual</t>
+        </is>
+      </c>
+      <c r="AY75" t="inlineStr">
+        <is>
+          <t>Midea MDHHU-MDHHS High Static Duct Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG75" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI75" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -14181,6 +15321,26 @@
           <t>MDLHU-H12B-2A__MO1HS-H12B-2A</t>
         </is>
       </c>
+      <c r="AT76" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU76" t="inlineStr">
+        <is>
+          <t>Midea Low Static Duct Service Manual</t>
+        </is>
+      </c>
+      <c r="AY76" t="inlineStr">
+        <is>
+          <t>Midea MDLHU Low Static Slim Duct Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG76" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI76" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -14372,6 +15532,26 @@
           <t>MDHHU-H18B-2A__MO1HS-H18B-2A</t>
         </is>
       </c>
+      <c r="AT77" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU77" t="inlineStr">
+        <is>
+          <t>Midea High Static Duct Service Manual</t>
+        </is>
+      </c>
+      <c r="AY77" t="inlineStr">
+        <is>
+          <t>Midea MDHHU-MDHHS High Static Duct Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG77" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI77" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -14563,6 +15743,26 @@
           <t>MDLHU-H18B-2A__MO1HS-H18B-2A</t>
         </is>
       </c>
+      <c r="AT78" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU78" t="inlineStr">
+        <is>
+          <t>Midea Low Static Duct Service Manual</t>
+        </is>
+      </c>
+      <c r="AY78" t="inlineStr">
+        <is>
+          <t>Midea MDLHU Low Static Slim Duct Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG78" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI78" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -14754,6 +15954,26 @@
           <t>MDHHU-H24B-2A__MO1HS-H24B-2A</t>
         </is>
       </c>
+      <c r="AT79" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU79" t="inlineStr">
+        <is>
+          <t>Midea High Static Duct Service Manual</t>
+        </is>
+      </c>
+      <c r="AY79" t="inlineStr">
+        <is>
+          <t>Midea MDHHU-MDHHS High Static Duct Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG79" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI79" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -14945,6 +16165,26 @@
           <t>MDHHS-H36B-2A__MO1HU-H36B-2A</t>
         </is>
       </c>
+      <c r="AT80" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU80" t="inlineStr">
+        <is>
+          <t>Midea High Static Duct Service Manual</t>
+        </is>
+      </c>
+      <c r="AY80" t="inlineStr">
+        <is>
+          <t>Midea MDHHU-MDHHS High Static Duct Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG80" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI80" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -15136,6 +16376,26 @@
           <t>MDHHS-H48B-2A__MO1HU-H48B-2A</t>
         </is>
       </c>
+      <c r="AT81" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU81" t="inlineStr">
+        <is>
+          <t>Midea High Static Duct Service Manual</t>
+        </is>
+      </c>
+      <c r="AY81" t="inlineStr">
+        <is>
+          <t>Midea MDHHU-MDHHS High Static Duct Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG81" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI81" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -15327,6 +16587,26 @@
           <t>MDHHS-H60B-2A__MO1HU-H60B-2A</t>
         </is>
       </c>
+      <c r="AT82" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU82" t="inlineStr">
+        <is>
+          <t>Midea High Static Duct Service Manual</t>
+        </is>
+      </c>
+      <c r="AY82" t="inlineStr">
+        <is>
+          <t>Midea MDHHU-MDHHS High Static Duct Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG82" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI82" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -15518,6 +16798,26 @@
           <t>MFAHU-H09B-2A__MO1ES-H09B-2A</t>
         </is>
       </c>
+      <c r="AT83" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU83" t="inlineStr">
+        <is>
+          <t>Midea Console Service Manual</t>
+        </is>
+      </c>
+      <c r="AY83" t="inlineStr">
+        <is>
+          <t>Midea MFAHU Floor Standing Console Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG83" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI83" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -15709,6 +17009,26 @@
           <t>MFAHU-H12B-2A__MO1ES-H12B-2A</t>
         </is>
       </c>
+      <c r="AT84" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU84" t="inlineStr">
+        <is>
+          <t>Midea Console Service Manual</t>
+        </is>
+      </c>
+      <c r="AY84" t="inlineStr">
+        <is>
+          <t>Midea MFAHU Floor Standing Console Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG84" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI84" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -15900,6 +17220,26 @@
           <t>MFAHU-H16B-2A__MO1ES-H18B-2A</t>
         </is>
       </c>
+      <c r="AT85" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU85" t="inlineStr">
+        <is>
+          <t>Midea Console Service Manual</t>
+        </is>
+      </c>
+      <c r="AY85" t="inlineStr">
+        <is>
+          <t>Midea MFAHU Floor Standing Console Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG85" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI85" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -16091,6 +17431,26 @@
           <t>MFAHU-H09B-2A__MO1HS-H09B-2A</t>
         </is>
       </c>
+      <c r="AT86" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU86" t="inlineStr">
+        <is>
+          <t>Midea Console Service Manual</t>
+        </is>
+      </c>
+      <c r="AY86" t="inlineStr">
+        <is>
+          <t>Midea MFAHU Floor Standing Console Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG86" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI86" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -16282,6 +17642,26 @@
           <t>MFAHU-H12B-2A__MO1HS-H12B-2A</t>
         </is>
       </c>
+      <c r="AT87" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU87" t="inlineStr">
+        <is>
+          <t>Midea Console Service Manual</t>
+        </is>
+      </c>
+      <c r="AY87" t="inlineStr">
+        <is>
+          <t>Midea MFAHU Floor Standing Console Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG87" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI87" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -16473,6 +17853,26 @@
           <t>MFAHU-H16B-2A__MO1HS-H18B-2A</t>
         </is>
       </c>
+      <c r="AT88" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU88" t="inlineStr">
+        <is>
+          <t>Midea Console Service Manual</t>
+        </is>
+      </c>
+      <c r="AY88" t="inlineStr">
+        <is>
+          <t>Midea MFAHU Floor Standing Console Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG88" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI88" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -16664,6 +18064,26 @@
           <t>MFBHU-H18B-2A__MO1ES-H18B-2A</t>
         </is>
       </c>
+      <c r="AT89" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU89" t="inlineStr">
+        <is>
+          <t>Midea Ceiling and Floor Service Manual</t>
+        </is>
+      </c>
+      <c r="AY89" t="inlineStr">
+        <is>
+          <t>Midea MFBHU-MFBHS Ceiling and Floor Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG89" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI89" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -16855,6 +18275,26 @@
           <t>MFBHU-H24B-2A__MO1ES-H24B-2A</t>
         </is>
       </c>
+      <c r="AT90" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU90" t="inlineStr">
+        <is>
+          <t>Midea Ceiling and Floor Service Manual</t>
+        </is>
+      </c>
+      <c r="AY90" t="inlineStr">
+        <is>
+          <t>Midea MFBHU-MFBHS Ceiling and Floor Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG90" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI90" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -17046,6 +18486,26 @@
           <t>MFBHS-H36B-2A__MO1BU-H36B-2A</t>
         </is>
       </c>
+      <c r="AT91" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU91" t="inlineStr">
+        <is>
+          <t>Midea Ceiling and Floor Service Manual</t>
+        </is>
+      </c>
+      <c r="AY91" t="inlineStr">
+        <is>
+          <t>Midea MFBHU-MFBHS Ceiling and Floor Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG91" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI91" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -17237,6 +18697,26 @@
           <t>MFBHS-H60B-2A__MO1BU-H60B-2A</t>
         </is>
       </c>
+      <c r="AT92" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU92" t="inlineStr">
+        <is>
+          <t>Midea Ceiling and Floor Service Manual</t>
+        </is>
+      </c>
+      <c r="AY92" t="inlineStr">
+        <is>
+          <t>Midea MFBHU-MFBHS Ceiling and Floor Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG92" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI92" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -17428,6 +18908,26 @@
           <t>MFBHU-H18B-2A__MO1HS-H18B-2A</t>
         </is>
       </c>
+      <c r="AT93" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU93" t="inlineStr">
+        <is>
+          <t>Midea Ceiling and Floor Service Manual</t>
+        </is>
+      </c>
+      <c r="AY93" t="inlineStr">
+        <is>
+          <t>Midea MFBHU-MFBHS Ceiling and Floor Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG93" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI93" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -17619,6 +19119,26 @@
           <t>MFBHU-H24B-2A__MO1HS-H24B-2A</t>
         </is>
       </c>
+      <c r="AT94" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU94" t="inlineStr">
+        <is>
+          <t>Midea Ceiling and Floor Service Manual</t>
+        </is>
+      </c>
+      <c r="AY94" t="inlineStr">
+        <is>
+          <t>Midea MFBHU-MFBHS Ceiling and Floor Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG94" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI94" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -17810,6 +19330,26 @@
           <t>MFBHS-H36B-2A__MO1HU-H36B-2A</t>
         </is>
       </c>
+      <c r="AT95" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU95" t="inlineStr">
+        <is>
+          <t>Midea Ceiling and Floor Service Manual</t>
+        </is>
+      </c>
+      <c r="AY95" t="inlineStr">
+        <is>
+          <t>Midea MFBHU-MFBHS Ceiling and Floor Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG95" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI95" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -18001,6 +19541,26 @@
           <t>MFBHS-H48B-2A__MO1HU-H48B-2A</t>
         </is>
       </c>
+      <c r="AT96" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU96" t="inlineStr">
+        <is>
+          <t>Midea Ceiling and Floor Service Manual</t>
+        </is>
+      </c>
+      <c r="AY96" t="inlineStr">
+        <is>
+          <t>Midea MFBHU-MFBHS Ceiling and Floor Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG96" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI96" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -18192,6 +19752,26 @@
           <t>MFBHS-H60B-2A__MO1HU-H60B-2A</t>
         </is>
       </c>
+      <c r="AT97" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU97" t="inlineStr">
+        <is>
+          <t>Midea Ceiling and Floor Service Manual</t>
+        </is>
+      </c>
+      <c r="AY97" t="inlineStr">
+        <is>
+          <t>Midea MFBHU-MFBHS Ceiling and Floor Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG97" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
+        </is>
+      </c>
       <c r="BI97" t="inlineStr">
         <is>
           <t>R-454B</t>
@@ -18381,6 +19961,26 @@
       <c r="AR98" t="inlineStr">
         <is>
           <t>MFBHS-H48B-2A__MO1BU-H48B-2A</t>
+        </is>
+      </c>
+      <c r="AT98" t="inlineStr">
+        <is>
+          <t>Midea Single-Zone Outdoor Unit Service Manual</t>
+        </is>
+      </c>
+      <c r="AU98" t="inlineStr">
+        <is>
+          <t>Midea Ceiling and Floor Service Manual</t>
+        </is>
+      </c>
+      <c r="AY98" t="inlineStr">
+        <is>
+          <t>Midea MFBHU-MFBHS Ceiling and Floor Installation Manual</t>
+        </is>
+      </c>
+      <c r="BG98" t="inlineStr">
+        <is>
+          <t>Midea Light Commercial Indoor Owners Manual</t>
         </is>
       </c>
       <c r="BI98" t="inlineStr">

</xml_diff>